<commit_message>
FEA: QR corrigidos das págs. 18, 23/61 e 64/68 e destinos confirmados
Cada artigo proposto foi conferido pelo conteúdo do PDF no Drive contra o
texto do box no livro. Os QR novos (PNG 900 px e SVG) foram relidos por
detector depois de gerados. A pág. 36 fica pendente: o artigo citado não
existe no Drive.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MsM8EmraRKzU1z7Ac7oN6i
</commit_message>
<xml_diff>
--- a/FEA-traducao-intercorrencias/FEA-Traducao-ES-Intercorrencias-Aulas-e-QR.xlsx
+++ b/FEA-traducao-intercorrencias/FEA-Traducao-ES-Intercorrencias-Aulas-e-QR.xlsx
@@ -1397,7 +1397,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Mudar o compartilhamento para «Qualquer pessoa com o link: leitor». Não mexe na arte, vale para PT e ES.</t>
+          <t>Abrir o arquivo no Drive &gt; Compartilhar &gt; Acesso geral: «Qualquer pessoa com o link», leitor. Não mexe na arte, vale para PT e ES.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>proposto https://drive.google.com/file/d/13rcR4MVX0frvJp3wgtFD1ko9IWQFiyco/view («ARTIGO 1 DELORENZI HIALU .pdf»)</t>
+          <t>https://drive.google.com/file/d/13rcR4MVX0frvJp3wgtFD1ko9IWQFiyco/view (CONFIRMADO: DeLorenzi, High Dose Pulsed Hyaluronidase · QR pronto: FEA-QR-pag18-HDPH-DeLorenzi)</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Mudar o compartilhamento para «Qualquer pessoa com o link: leitor». Não mexe na arte, vale para PT e ES.</t>
+          <t>Abrir o arquivo no Drive &gt; Compartilhar &gt; Acesso geral: «Qualquer pessoa com o link», leitor. Não mexe na arte, vale para PT e ES.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>proposto https://drive.google.com/file/d/1IQ-osnYyMdlCR511_SwOqVRdPjxqD3AI/view</t>
+          <t>https://drive.google.com/file/d/1IQ-osnYyMdlCR511_SwOqVRdPjxqD3AI/view (CONFIRMADO: Mehta et al. 2022 · QR pronto: FEA-QR-pag23-e-61)</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Mudar o compartilhamento para «Qualquer pessoa com o link: leitor». Não mexe na arte, vale para PT e ES.</t>
+          <t>Abrir o arquivo no Drive &gt; Compartilhar &gt; Acesso geral: «Qualquer pessoa com o link», leitor. Não mexe na arte, vale para PT e ES.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Mudar o compartilhamento para «Qualquer pessoa com o link: leitor». Não mexe na arte, vale para PT e ES.</t>
+          <t>Abrir o arquivo no Drive &gt; Compartilhar &gt; Acesso geral: «Qualquer pessoa com o link», leitor. Não mexe na arte, vale para PT e ES.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Mudar o compartilhamento para «Qualquer pessoa com o link: leitor». Não mexe na arte, vale para PT e ES.</t>
+          <t>Abrir o arquivo no Drive &gt; Compartilhar &gt; Acesso geral: «Qualquer pessoa com o link», leitor. Não mexe na arte, vale para PT e ES.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>proposto https://drive.google.com/file/d/1g2G9VADj6u5qsG5G1Zwqv_0kcow2-Zgb/view («2. ARTIGO delorenzi2014.pdf»)</t>
+          <t>FALTA O ARQUIVO: o box cita «Consensus Guidelines for the Management of HA Filler-Induced Vascular Occlusion», que não está no Drive (o delorenzi2014 é outro artigo). Subir o PDF na pasta de artigos.</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Mudar o compartilhamento para «Qualquer pessoa com o link: leitor». Não mexe na arte, vale para PT e ES.</t>
+          <t>Abrir o arquivo no Drive &gt; Compartilhar &gt; Acesso geral: «Qualquer pessoa com o link», leitor. Não mexe na arte, vale para PT e ES.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>proposto https://drive.google.com/file/d/1IQ-osnYyMdlCR511_SwOqVRdPjxqD3AI/view</t>
+          <t>https://drive.google.com/file/d/1IQ-osnYyMdlCR511_SwOqVRdPjxqD3AI/view (CONFIRMADO · QR pronto: FEA-QR-pag23-e-61)</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>proposto https://drive.google.com/file/d/1DLM3QIm8ui-37tXlv33AazCSiK57hIgP/view (Kim et al., J Korean Med Sci 2015)</t>
+          <t>https://drive.google.com/file/d/1DLM3QIm8ui-37tXlv33AazCSiK57hIgP/view (CONFIRMADO: Kim et al., J Korean Med Sci 2015 · QR pronto: FEA-QR-pag64-e-68)</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -2326,12 +2326,12 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>André Vivas (arte) · equipe médica confirma se é o mesmo artigo da pág. 64</t>
+          <t>André Vivas (arte)</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>proposto https://drive.google.com/file/d/1DLM3QIm8ui-37tXlv33AazCSiK57hIgP/view</t>
+          <t>https://drive.google.com/file/d/1DLM3QIm8ui-37tXlv33AazCSiK57hIgP/view (CONFIRMADO: mesmo artigo da pág. 64 · QR pronto: FEA-QR-pag64-e-68)</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -2602,22 +2602,22 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Págs. 64 e 68</t>
+          <t>Artigo da pág. 36</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Usam o mesmo QR, mas os textos descrevem estudos diferentes (oftálmico vs. cerebral). Confirmar se é o mesmo artigo.</t>
+          <t>Subir o PDF do «Consensus Guidelines for the Management of Hyaluronic Acid Filler-Induced Vascular Occlusion» citado no box. Não existe no Drive.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Equipe médica (Francine)</t>
+          <t>Keila / equipe médica</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Não trava o PDF</t>
+          <t>Só o QR da pág. 36</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
FEA intercorrências ES: tradução completa, revisão cega aplicada e pipeline de produção do PDF
- traducao/: 6 partes PT/ES, relatórios e decisões comuns
- revisao/: revisão cega fea-revision-es (6 partes LIBERADAS, zero classe A)
- produccion/: mapa id→ES, scripts de display, arte, rótulos, fontes, OCR, layout, QR e ficha de entrega
- traduzir_pdf: itens de lista separados pelo marcador, colunas de quadro, hifenização, pílulas
- planilha de aulas e QR atualizada com os links decodificados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MsM8EmraRKzU1z7Ac7oN6i
</commit_message>
<xml_diff>
--- a/FEA-traducao-intercorrencias/FEA-Traducao-ES-Intercorrencias-Aulas-e-QR.xlsx
+++ b/FEA-traducao-intercorrencias/FEA-Traducao-ES-Intercorrencias-Aulas-e-QR.xlsx
@@ -525,12 +525,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>≈ 40 mil</t>
+          <t>36.081</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Estimativa: as págs. 1 a 80 têm 15,5 mil palavras. Número exato sai na Passagem 0 com o PDF.</t>
+          <t>Contagem exata da camada de texto do PDF (fora o texto embutido em arte: capa, aberturas e 4 figuras, também traduzidos).</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Quando os links das aulas dubladas existirem. ~2 h de trabalho depois que os links chegarem.</t>
+          <t>Na entrega v1 os QR de aula abrem a aula em PT. Quando os links das aulas dubladas existirem: ~2 h de trabalho.</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Págs. 18, 23, 36, 61, 64 e 68: exigem QR novo na arte (PT e ES).</t>
+          <t>Págs. 18, 23, 36, 61, 64 e 68. Na versão ES, 5 já foram regerados com o destino confirmado; falta só a 36 (arquivo do artigo inexistente). O PT continua com o erro até o André trocar.</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -669,12 +669,12 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>½ dia</t>
+          <t>feito</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Dia 1 · esta planilha é atualizada com as páginas exatas</t>
+          <t>05/10/2026</t>
         </is>
       </c>
     </row>
@@ -686,12 +686,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>2 a 3 dias</t>
+          <t>feito</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Dias 1 a 3</t>
+          <t>05/10/2026</t>
         </is>
       </c>
     </row>
@@ -703,12 +703,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2 a 3 dias</t>
+          <t>feito</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Dias 3 a 6</t>
+          <t>05/10/2026</t>
         </is>
       </c>
     </row>
@@ -720,12 +720,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>1 dia</t>
+          <t>feito</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Dias 6 e 7</t>
+          <t>05/10/2026 · 6 partes LIBERADAS, zero achado clínico</t>
         </is>
       </c>
     </row>
@@ -737,12 +737,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>5 a 7 dias úteis</t>
+          <t>feito</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Se o PDF for liberado hoje (05/10): entre 12 e 14/10/2026, com os QR de aula ainda em PT</t>
+          <t>05/10/2026, com os QR de aula ainda em PT</t>
         </is>
       </c>
     </row>
@@ -865,14 +865,10 @@
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr"/>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>conferir na Passagem 0</t>
-        </is>
-      </c>
+      <c r="H2" s="5" t="inlineStr"/>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>pendente</t>
+          <t>pendente (aula dublada)</t>
         </is>
       </c>
     </row>
@@ -906,14 +902,10 @@
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>conferir na Passagem 0</t>
-        </is>
-      </c>
+      <c r="H3" s="5" t="inlineStr"/>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>pendente</t>
+          <t>pendente (aula dublada)</t>
         </is>
       </c>
     </row>
@@ -923,7 +915,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>~32</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -943,18 +935,14 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>a decodificar do PDF</t>
+          <t>https://www.youtube.com/watch?v=zb0ZWo29Pk8</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>conferir na Passagem 0</t>
-        </is>
-      </c>
+      <c r="H4" s="5" t="inlineStr"/>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>pendente</t>
+          <t>pendente (aula dublada)</t>
         </is>
       </c>
     </row>
@@ -964,7 +952,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>~35</t>
+          <t>35</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -984,18 +972,14 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>a decodificar do PDF</t>
+          <t>https://www.youtube.com/watch?v=w7ZawtnNb2o</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>conferir na Passagem 0</t>
-        </is>
-      </c>
+      <c r="H5" s="5" t="inlineStr"/>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>pendente</t>
+          <t>pendente (aula dublada)</t>
         </is>
       </c>
     </row>
@@ -1029,14 +1013,10 @@
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>conferir na Passagem 0</t>
-        </is>
-      </c>
+      <c r="H6" s="5" t="inlineStr"/>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>pendente</t>
+          <t>pendente (aula dublada)</t>
         </is>
       </c>
     </row>
@@ -1070,14 +1050,10 @@
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>conferir na Passagem 0</t>
-        </is>
-      </c>
+      <c r="H7" s="5" t="inlineStr"/>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>pendente</t>
+          <t>pendente (aula dublada)</t>
         </is>
       </c>
     </row>
@@ -1111,14 +1087,10 @@
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr"/>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>conferir na Passagem 0</t>
-        </is>
-      </c>
+      <c r="H8" s="5" t="inlineStr"/>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>pendente</t>
+          <t>pendente (aula dublada)</t>
         </is>
       </c>
     </row>
@@ -1152,14 +1124,10 @@
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>conferir na Passagem 0</t>
-        </is>
-      </c>
+      <c r="H9" s="5" t="inlineStr"/>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>pendente</t>
+          <t>pendente (aula dublada)</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1137,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>~74</t>
+          <t>74</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1189,18 +1157,14 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>a decodificar do PDF</t>
+          <t>https://www.youtube.com/watch?v=YUirUEfaMjc</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr"/>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>conferir na Passagem 0</t>
-        </is>
-      </c>
+      <c r="H10" s="5" t="inlineStr"/>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>pendente</t>
+          <t>pendente (aula dublada)</t>
         </is>
       </c>
     </row>
@@ -1225,23 +1189,19 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Intercorrências e emergências médicas · Complicações isquêmicas agudas</t>
+          <t>Intercorrências e emergências médicas · Complicações agudas não isquêmicas · confirmar</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>a decodificar do PDF</t>
+          <t>https://www.youtube.com/watch?v=XzONB5671uY</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>conferir na Passagem 0</t>
-        </is>
-      </c>
+      <c r="H11" s="5" t="inlineStr"/>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>pendente</t>
+          <t>pendente (aula dublada)</t>
         </is>
       </c>
     </row>
@@ -1266,23 +1226,19 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Intercorrências e emergências médicas · Complicações isquêmicas agudas</t>
+          <t>Intercorrências e emergências médicas · Complicações agudas não isquêmicas · confirmar</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>a decodificar do PDF</t>
+          <t>https://www.youtube.com/watch?v=dh26SwtfD2U</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr"/>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>conferir na Passagem 0</t>
-        </is>
-      </c>
+      <c r="H12" s="5" t="inlineStr"/>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>pendente</t>
+          <t>pendente (aula dublada)</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1464,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Corrigir junto, já com o link do artigo; não traduz</t>
+          <t>FEITO na versão ES: QR regerado para o artigo HDPH</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
@@ -1535,7 +1491,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>provável https://drive.google.com/file/d/1F8aLFw8VV62JQngjfkHLNpHn2lr8jmjj/view</t>
+          <t>https://drive.google.com/file/d/1F8aLFw8VV62JQngjfkHLNpHn2lr8jmjj/view</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -1555,7 +1511,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>provável https://drive.google.com/file/d/1F8aLFw8VV62JQngjfkHLNpHn2lr8jmjj/view</t>
+          <t>https://drive.google.com/file/d/1F8aLFw8VV62JQngjfkHLNpHn2lr8jmjj/view</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -1612,7 +1568,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Corrigir junto; não traduz</t>
+          <t>FEITO na versão ES: QR regerado (exceto pág. 36, falta o arquivo)</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -1639,7 +1595,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>provável https://drive.google.com/file/d/1F8aLFw8VV62JQngjfkHLNpHn2lr8jmjj/view</t>
+          <t>https://drive.google.com/file/d/1F8aLFw8VV62JQngjfkHLNpHn2lr8jmjj/view</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1659,7 +1615,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>provável https://drive.google.com/file/d/1F8aLFw8VV62JQngjfkHLNpHn2lr8jmjj/view</t>
+          <t>https://drive.google.com/file/d/1F8aLFw8VV62JQngjfkHLNpHn2lr8jmjj/view</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -1772,7 +1728,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>~32</t>
+          <t>32</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1787,7 +1743,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>a decodificar do PDF</t>
+          <t>https://www.youtube.com/watch?v=zb0ZWo29Pk8</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -1831,7 +1787,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>provável https://drive.google.com/file/d/19A8eYYAofI8Eiq4fIyk0kv-kJZf8aAvM/view</t>
+          <t>https://drive.google.com/file/d/19A8eYYAofI8Eiq4fIyk0kv-kJZf8aAvM/view</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1851,7 +1807,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>provável https://drive.google.com/file/d/19A8eYYAofI8Eiq4fIyk0kv-kJZf8aAvM/view</t>
+          <t>https://drive.google.com/file/d/19A8eYYAofI8Eiq4fIyk0kv-kJZf8aAvM/view</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1868,7 +1824,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>~35</t>
+          <t>35</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1883,7 +1839,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>a decodificar do PDF</t>
+          <t>https://www.youtube.com/watch?v=w7ZawtnNb2o</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1927,7 +1883,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>a decodificar do PDF</t>
+          <t>https://drive.google.com/file/d/11p9QK_qVuG__8htGvDWr3wPImLY-Ovbp/view</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -1952,7 +1908,7 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Corrigir junto; não traduz</t>
+          <t>FEITO na versão ES: QR regerado (exceto pág. 36, falta o arquivo)</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
@@ -2188,7 +2144,7 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Corrigir junto; não traduz</t>
+          <t>FEITO na versão ES: QR regerado (exceto pág. 36, falta o arquivo)</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
@@ -2284,7 +2240,7 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Corrigir junto; não traduz</t>
+          <t>FEITO na versão ES: QR regerado (exceto pág. 36, falta o arquivo)</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
@@ -2336,7 +2292,7 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Corrigir junto; não traduz</t>
+          <t>FEITO na versão ES: QR regerado (exceto pág. 36, falta o arquivo)</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
@@ -2348,7 +2304,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>~74</t>
+          <t>74</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -2363,7 +2319,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>a decodificar do PDF</t>
+          <t>https://www.youtube.com/watch?v=YUirUEfaMjc</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -2407,7 +2363,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>a decodificar do PDF</t>
+          <t>https://www.youtube.com/watch?v=XzONB5671uY</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -2451,7 +2407,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>a decodificar do PDF</t>
+          <t>https://www.youtube.com/watch?v=dh26SwtfD2U</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -2493,7 +2449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2533,12 +2489,12 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Acesso ao PDF original</t>
+          <t>Aulas dubladas</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>O arquivo tem 28 MB e a rede deste ambiente bloqueia o download direto do Drive (o conector só baixa até 10 MB). Liberar os domínios do Google no ambiente, ou subir o PDF em partes menores que 10 MB.</t>
+          <t>Confirmar se as 11 aulas serão dubladas e publicadas no YouTube como não listadas, como no ebook de olheiras (18 aulas). A produção das aulas é da FEA, fora do escopo da skill.</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -2548,7 +2504,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Trava o início da tradução</t>
+          <t>Não trava o PDF</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr"/>
@@ -2556,17 +2512,17 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Aulas dubladas</t>
+          <t>Corrigir os 6 QR com ERRO no PT</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Confirmar se as 11 aulas serão dubladas e publicadas no YouTube como não listadas, como no ebook de olheiras (18 aulas). A produção das aulas é da FEA, fora do escopo da skill.</t>
+          <t>Recomendação: corrigir o original PT (André) e eu aplico os mesmos destinos na versão ES. Os links propostos estão na aba «QR para ajustar».</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Keila</t>
+          <t>Keila + equipe médica</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -2579,22 +2535,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Corrigir os 6 QR com ERRO no PT</t>
+          <t>Artigo da pág. 36</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Recomendação: corrigir o original PT (André) e eu aplico os mesmos destinos na versão ES. Os links propostos estão na aba «QR para ajustar».</t>
+          <t>Subir o PDF do «Consensus Guidelines for the Management of Hyaluronic Acid Filler-Induced Vascular Occlusion» citado no box. Não existe no Drive.</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Keila + equipe médica</t>
+          <t>Keila / equipe médica</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Não trava o PDF</t>
+          <t>Só o QR da pág. 36</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr"/>
@@ -2602,22 +2558,22 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Artigo da pág. 36</t>
+          <t>Numeração dos vídeos</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Subir o PDF do «Consensus Guidelines for the Management of Hyaluronic Acid Filler-Induced Vascular Occlusion» citado no box. Não existe no Drive.</t>
+          <t>Só os 3 últimos boxes têm número (Vídeo 9, 10 e 11). Padronizar no ES: todos numerados ou nenhum. Recomendação: numerar todos de 1 a 11.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Keila / equipe médica</t>
+          <t>Keila</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Só o QR da pág. 36</t>
+          <t>Não trava o PDF</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
@@ -2625,12 +2581,12 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Numeração dos vídeos</t>
+          <t>Título do livro em espanhol</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Só os 3 últimos boxes têm número (Vídeo 9, 10 e 11). Padronizar no ES: todos numerados ou nenhum. Recomendação: numerar todos de 1 a 11.</t>
+          <t>Proposta: «Intercurrencias en el relleno con ácido hialurónico: diagnóstico y conductas clínicas ante complicaciones estéticas» (mantém «Intercurrencias», como na sigla ARTI do ebook de olheiras).</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -2648,22 +2604,22 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Título do livro em espanhol</t>
+          <t>Autor · tempo de reperfusão capilar (pág. 27)</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Proposta: «Intercurrencias en el relleno con ácido hialurónico: diagnóstico y conductas clínicas ante complicaciones estéticas» (mantém «Intercurrencias», como na sigla ARTI do ebook de olheiras).</t>
+          <t>O PT diz «redução do tempo de reperfusão capilar» como sinal de isquemia; o correto é aumento (lentificação), como na pág. 14. O ES espelhou o original.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Keila</t>
+          <t>Dr. João / equipe médica</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Não trava o PDF</t>
+          <t>Prioridade clínica</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr"/>
@@ -2671,25 +2627,163 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>Autor · dose da hialuronidase (págs. 31, 41, 50)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>«Injetar 1.000 UTR/mL» informa a concentração, não a dose nem o volume.</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Dr. João / equipe médica</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Prioridade clínica</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Autor · piperacilina</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>4,5 g num capítulo e 3,375 g em outro.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Equipe médica</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Prioridade clínica</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Autor · janela da retina</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Quatro números diferentes para a janela de tempo da retina (30 min, 90 min, 4 h, 12 h) ao longo do livro.</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Equipe médica</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Revisar PT e ES</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Autor · figuras com título repetido</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Fig. 5, 27, 31 (legenda copiada da 30), 36, 43 repetido nas 44 e 45, 62 (Tyndall).</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>André Vivas + equipe médica</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Revisar PT e ES</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Linha vermelha 7 · imagens geradas por IA</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Figuras 37, 39, 41, 52, 53, 61 e 62 declaram imagem criada ou adaptada por IA; a 53 vem de «busca na internet» (direito de uso).</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Keila + Dr. João</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Decisão editorial</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Autor · conceitos técnicos</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Er:YAG listado como «não ablativo»; Tyndall explicado como «refração»/«sombra»; triamcinolona «diluída» sem concentração final.</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Equipe médica</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Revisar PT e ES</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
           <t>Artigos científicos</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Pela regra da skill, os 12 QR de artigo (contando a pág. 18 corrigida) ficam em inglês e com o mesmo link na versão ES.</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Informativo</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Nenhum</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
FEA intercorrências ES: aba Subir no YouTube com as 11 aulas dubladas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MsM8EmraRKzU1z7Ac7oN6i
</commit_message>
<xml_diff>
--- a/FEA-traducao-intercorrencias/FEA-Traducao-ES-Intercorrencias-Aulas-e-QR.xlsx
+++ b/FEA-traducao-intercorrencias/FEA-Traducao-ES-Intercorrencias-Aulas-e-QR.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Resumo e prazo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Aulas para traduzir" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="QR para ajustar" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Decisões pendentes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Subir no YouTube" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Aulas para traduzir" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="QR para ajustar" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Decisões pendentes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +37,11 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="005B4599"/>
+      <sz val="13"/>
     </font>
     <font>
       <b val="1"/>
@@ -77,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -89,13 +95,14 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -774,6 +781,651 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Subir as 11 aulas dubladas no YouTube do Dr. João como NÃO LISTADO · traduções prontas no HeyGen (05/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1. Entrar no HeyGen &gt; Video Translate e baixar o vídeo pelo «Arquivo no HeyGen» (coluna D). Conferir pelo ID (coluna F) se houver dois com o mesmo nome: use sempre o que está «Completed».</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2. Abrir studio.youtube.com no canal do Dr. João &gt; Criar &gt; Enviar vídeos &gt; escolher o arquivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3. Título: copiar a coluna C. Descrição: copiar a coluna G.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4. Público: «Não, não é conteúdo para crianças». Em «Restrição de idade», marcar +18 só onde a coluna H diz SIM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5. Visibilidade: NÃO LISTADO (nunca Público). Salvar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6. Copiar o link do vídeo (youtu.be/...) e colar na coluna I. Mudar o status (coluna J) para «subido».</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>7. Quando os 11 links estiverem preenchidos, avisar a Keila: os QR do livro são regerados com esses links.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Nº</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Página do livro</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Título no YouTube (copiar)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo no HeyGen (baixar)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Duração</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>ID da tradução no HeyGen</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Descrição no YouTube (copiar)</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Restrição de idade +18</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Link do YouTube (colar aqui)</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Introducción al razonamiento clínico de las complicaciones agudas isquémicas</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Introducción al razonamiento clínico de complicaciones agudas isquémicas-Spanish</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>24 min</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>42d9570604e04b26a5c18c76e870e752-es</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Clase complementaria del libro «Intercurrencias en el relleno con ácido hialurónico» (Dr. João Pithon), pág. 15. Versión doblada al español. Contenido técnico dirigido exclusivamente a profesionales de la salud habilitados.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>a subir</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Revisión anatómica global de la cara: vascularización</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Revisión anatómica global de la cara - Vascularización-Spanish</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>8 min</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>03157b737e2e45ba86d5e666477f8ca6-es</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Clase complementaria del libro «Intercurrencias en el relleno con ácido hialurónico» (Dr. João Pithon), pág. 29. Versión doblada al español. Contenido técnico dirigido exclusivamente a profesionales de la salud habilitados.</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>SIM (o original tem)</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>a subir</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Hialuronidasa</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Hialuronidasa-Spanish</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>33 min</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>2d367ed2ac5a4d10bfb057cf2aae161e-es</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Clase complementaria del libro «Intercurrencias en el relleno con ácido hialurónico» (Dr. João Pithon), pág. 32. Versión doblada al español. Contenido técnico dirigido exclusivamente a profesionales de la salud habilitados.</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>a subir</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Rinomodelación: protocolo y manejo de las complicaciones</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Rinomodelación - Protocolo y manejo de las complicaciones-Spanish</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>18 min</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>0e6164337eb241569e406756c4160473-es</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Clase complementaria del libro «Intercurrencias en el relleno con ácido hialurónico» (Dr. João Pithon), pág. 35. Versión doblada al español. Contenido técnico dirigido exclusivamente a profesionales de la salud habilitados.</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>a subir</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Mecanismos de seguridad con cánulas</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Mecanismos de seguridad con cánulas-Spanish</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>13 min</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>a43ff9f20cbe4820941374cd40e5565e-es</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Clase complementaria del libro «Intercurrencias en el relleno con ácido hialurónico» (Dr. João Pithon), pág. 37. Versión doblada al español. Contenido técnico dirigido exclusivamente a profesionales de la salud habilitados.</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>a subir</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Rinomodelación: ¿aguja o cánula?</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Rinomodelación - ¿Aguja o cánula?-Spanish</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>8 min</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>1c83fc523f364de69e4982b244ba8f5a-es</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Clase complementaria del libro «Intercurrencias en el relleno con ácido hialurónico» (Dr. João Pithon), pág. 43. Versión doblada al español. Contenido técnico dirigido exclusivamente a profesionales de la salud habilitados.</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr"/>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>a subir</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Relleno full face guiado por ecografía, en vivo</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Relleno full face guiado por ultrasonido en vivo-Spanish</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>54 min</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>f5844178d1284bc0954a19dd5a33869e-es</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Clase complementaria del libro «Intercurrencias en el relleno con ácido hialurónico» (Dr. João Pithon), pág. 45. Versión doblada al español. Contenido técnico dirigido exclusivamente a profesionales de la salud habilitados.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>a subir</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Amaurosis: protocolo de manejo de las complicaciones</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Amaurosis - Protocolo de manejo de las complicaciones-Spanish</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>13 min</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>0b84b17b226a46f9a2a7c4af575e44e7-es</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Clase complementaria del libro «Intercurrencias en el relleno con ácido hialurónico» (Dr. João Pithon), pág. 63. Versión doblada al español. Contenido técnico dirigido exclusivamente a profesionales de la salud habilitados.</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr"/>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>a subir</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Complejo vascular nasoglabelar</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Complejo vascular nasoglabelar-Spanish</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>11 min</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>a309a29b82db4e82a96550ac5783a21d-es</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Clase complementaria del libro «Intercurrencias en el relleno con ácido hialurónico» (Dr. João Pithon), pág. 74. Versión doblada al español. Contenido técnico dirigido exclusivamente a profesionales de la salud habilitados.</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>SIM (o original tem)</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr"/>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>a subir</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Complicaciones agudas no isquémicas (parte 1)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Complicaciones agudas no isquémicas - Parte 1-Spanish</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>6 min</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>77452f298fb044e59a615c505cb5b71d-es</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Clase complementaria del libro «Intercurrencias en el relleno con ácido hialurónico» (Dr. João Pithon), pág. 79. Versión doblada al español. Contenido técnico dirigido exclusivamente a profesionales de la salud habilitados.</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr"/>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>a subir</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Complicaciones agudas no isquémicas (parte 2)</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Complicaciones agudas no isquémicas - Parte 2-Spanish</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>6 min</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>d8499de7f6284f4b80a5d5557dc4625e-es</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Clase complementaria del libro «Intercurrencias en el relleno con ácido hialurónico» (Dr. João Pithon), pág. 80. Versión doblada al español. Contenido técnico dirigido exclusivamente a profesionales de la salud habilitados.</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr"/>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>a subir</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="J11:J21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"a subir,subido,QR atualizado"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -864,11 +1516,15 @@
           <t>https://www.youtube.com/watch?v=HW62ZM3NDC8</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr"/>
-      <c r="H2" s="5" t="inlineStr"/>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>pendente (aula dublada)</t>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>ver aba «Subir no YouTube»</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr"/>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>pronto</t>
         </is>
       </c>
     </row>
@@ -901,11 +1557,15 @@
           <t>https://www.youtube.com/watch?v=2Qoh7fWG5w4</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>pendente (aula dublada)</t>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>ver aba «Subir no YouTube»</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr"/>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>pronto</t>
         </is>
       </c>
     </row>
@@ -938,11 +1598,15 @@
           <t>https://www.youtube.com/watch?v=zb0ZWo29Pk8</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr"/>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>pendente (aula dublada)</t>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>ver aba «Subir no YouTube»</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>pronto</t>
         </is>
       </c>
     </row>
@@ -975,11 +1639,15 @@
           <t>https://www.youtube.com/watch?v=w7ZawtnNb2o</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>pendente (aula dublada)</t>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>ver aba «Subir no YouTube»</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>pronto</t>
         </is>
       </c>
     </row>
@@ -1012,11 +1680,15 @@
           <t>https://www.youtube.com/watch?v=_yWZEknxYqo</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>pendente (aula dublada)</t>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>ver aba «Subir no YouTube»</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>pronto</t>
         </is>
       </c>
     </row>
@@ -1049,11 +1721,15 @@
           <t>https://www.youtube.com/watch?v=NCHkXFLKZds</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>pendente (aula dublada)</t>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>ver aba «Subir no YouTube»</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>pronto</t>
         </is>
       </c>
     </row>
@@ -1086,11 +1762,15 @@
           <t>https://www.youtube.com/watch?v=QocyeCsLs9M</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr"/>
-      <c r="H8" s="5" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>pendente (aula dublada)</t>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>ver aba «Subir no YouTube»</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr"/>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>pronto</t>
         </is>
       </c>
     </row>
@@ -1123,11 +1803,15 @@
           <t>https://www.youtube.com/watch?v=GnGMUiPcoC0</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr"/>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>pendente (aula dublada)</t>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>ver aba «Subir no YouTube»</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>pronto</t>
         </is>
       </c>
     </row>
@@ -1160,11 +1844,15 @@
           <t>https://www.youtube.com/watch?v=YUirUEfaMjc</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr"/>
-      <c r="H10" s="5" t="inlineStr"/>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>pendente (aula dublada)</t>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>ver aba «Subir no YouTube»</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>pronto</t>
         </is>
       </c>
     </row>
@@ -1197,11 +1885,15 @@
           <t>https://www.youtube.com/watch?v=XzONB5671uY</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr"/>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>pendente (aula dublada)</t>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>ver aba «Subir no YouTube»</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>pronto</t>
         </is>
       </c>
     </row>
@@ -1234,25 +1926,29 @@
           <t>https://www.youtube.com/watch?v=dh26SwtfD2U</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr"/>
-      <c r="H12" s="5" t="inlineStr"/>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>pendente (aula dublada)</t>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>ver aba «Subir no YouTube»</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>pronto</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="I2:I12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"pendente,em produção,pronto"</formula1>
+      <formula1>"pendente,em produção,pronto,QR atualizado"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1371,7 +2067,7 @@
           <t>Não traduz (artigo científico fica em inglês, link igual)</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -1410,12 +2106,12 @@
       </c>
       <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Regerar QR para a aula dublada quando o link ES existir</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -1467,7 +2163,7 @@
           <t>FEITO na versão ES: QR regerado para o artigo HDPH</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -1519,7 +2215,7 @@
           <t>Não traduz (artigo científico fica em inglês, link igual)</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -1571,7 +2267,7 @@
           <t>FEITO na versão ES: QR regerado (exceto pág. 36, falta o arquivo)</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -1623,7 +2319,7 @@
           <t>Não traduz (artigo científico fica em inglês, link igual)</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -1662,12 +2358,12 @@
       </c>
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>Regerar QR para a aula dublada quando o link ES existir</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -1719,7 +2415,7 @@
           <t>Não traduz (artigo científico fica em inglês, link igual)</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -1758,12 +2454,12 @@
       </c>
       <c r="G10" s="3" t="inlineStr"/>
       <c r="H10" s="3" t="inlineStr"/>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="I10" s="8" t="inlineStr">
         <is>
           <t>Regerar QR para a aula dublada quando o link ES existir</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -1815,7 +2511,7 @@
           <t>Não traduz (artigo científico fica em inglês, link igual)</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -1854,12 +2550,12 @@
       </c>
       <c r="G12" s="3" t="inlineStr"/>
       <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Regerar QR para a aula dublada quando o link ES existir</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -1911,7 +2607,7 @@
           <t>FEITO na versão ES: QR regerado (exceto pág. 36, falta o arquivo)</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -1950,12 +2646,12 @@
       </c>
       <c r="G14" s="3" t="inlineStr"/>
       <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="6" t="inlineStr">
+      <c r="I14" s="8" t="inlineStr">
         <is>
           <t>Regerar QR para a aula dublada quando o link ES existir</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -2007,7 +2703,7 @@
           <t>Não traduz (artigo científico fica em inglês, link igual)</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -2046,12 +2742,12 @@
       </c>
       <c r="G16" s="3" t="inlineStr"/>
       <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="I16" s="8" t="inlineStr">
         <is>
           <t>Regerar QR para a aula dublada quando o link ES existir</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -2090,12 +2786,12 @@
       </c>
       <c r="G17" s="3" t="inlineStr"/>
       <c r="H17" s="3" t="inlineStr"/>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="I17" s="8" t="inlineStr">
         <is>
           <t>Regerar QR para a aula dublada quando o link ES existir</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -2147,7 +2843,7 @@
           <t>FEITO na versão ES: QR regerado (exceto pág. 36, falta o arquivo)</t>
         </is>
       </c>
-      <c r="J18" s="5" t="inlineStr">
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -2186,12 +2882,12 @@
       </c>
       <c r="G19" s="3" t="inlineStr"/>
       <c r="H19" s="3" t="inlineStr"/>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t>Regerar QR para a aula dublada quando o link ES existir</t>
         </is>
       </c>
-      <c r="J19" s="5" t="inlineStr">
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -2243,7 +2939,7 @@
           <t>FEITO na versão ES: QR regerado (exceto pág. 36, falta o arquivo)</t>
         </is>
       </c>
-      <c r="J20" s="5" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -2295,7 +2991,7 @@
           <t>FEITO na versão ES: QR regerado (exceto pág. 36, falta o arquivo)</t>
         </is>
       </c>
-      <c r="J21" s="5" t="inlineStr">
+      <c r="J21" s="6" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -2334,12 +3030,12 @@
       </c>
       <c r="G22" s="3" t="inlineStr"/>
       <c r="H22" s="3" t="inlineStr"/>
-      <c r="I22" s="6" t="inlineStr">
+      <c r="I22" s="8" t="inlineStr">
         <is>
           <t>Regerar QR para a aula dublada quando o link ES existir</t>
         </is>
       </c>
-      <c r="J22" s="5" t="inlineStr">
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -2378,12 +3074,12 @@
       </c>
       <c r="G23" s="3" t="inlineStr"/>
       <c r="H23" s="3" t="inlineStr"/>
-      <c r="I23" s="6" t="inlineStr">
+      <c r="I23" s="8" t="inlineStr">
         <is>
           <t>Regerar QR para a aula dublada quando o link ES existir</t>
         </is>
       </c>
-      <c r="J23" s="5" t="inlineStr">
+      <c r="J23" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -2422,12 +3118,12 @@
       </c>
       <c r="G24" s="3" t="inlineStr"/>
       <c r="H24" s="3" t="inlineStr"/>
-      <c r="I24" s="6" t="inlineStr">
+      <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Regerar QR para a aula dublada quando o link ES existir</t>
         </is>
       </c>
-      <c r="J24" s="5" t="inlineStr">
+      <c r="J24" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -2443,7 +3139,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2507,7 +3203,7 @@
           <t>Não trava o PDF</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -2530,7 +3226,7 @@
           <t>Não trava o PDF</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr"/>
+      <c r="E3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -2553,7 +3249,7 @@
           <t>Só o QR da pág. 36</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2576,7 +3272,7 @@
           <t>Não trava o PDF</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2599,7 +3295,7 @@
           <t>Não trava o PDF</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr"/>
+      <c r="E6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -2622,7 +3318,7 @@
           <t>Prioridade clínica</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -2645,7 +3341,7 @@
           <t>Prioridade clínica</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr"/>
+      <c r="E8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -2668,7 +3364,7 @@
           <t>Prioridade clínica</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr"/>
+      <c r="E9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -2691,7 +3387,7 @@
           <t>Revisar PT e ES</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr"/>
+      <c r="E10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -2714,7 +3410,7 @@
           <t>Revisar PT e ES</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -2737,7 +3433,7 @@
           <t>Decisão editorial</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr"/>
+      <c r="E12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2760,7 +3456,7 @@
           <t>Revisar PT e ES</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr"/>
+      <c r="E13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2783,7 +3479,7 @@
           <t>Nenhum</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr"/>
+      <c r="E14" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
FEA intercorrências ES: QR das 11 aulas para o YouTube ES, cabeçalho oculto removido, rodada 2 da revisão
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MsM8EmraRKzU1z7Ac7oN6i
</commit_message>
<xml_diff>
--- a/FEA-traducao-intercorrencias/FEA-Traducao-ES-Intercorrencias-Aulas-e-QR.xlsx
+++ b/FEA-traducao-intercorrencias/FEA-Traducao-ES-Intercorrencias-Aulas-e-QR.xlsx
@@ -799,7 +799,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Subir as 11 aulas dubladas no YouTube do Dr. João como NÃO LISTADO · traduções prontas no HeyGen (05/10/2026)</t>
+          <t>11 aulas dubladas no YouTube do Dr. João como NÃO LISTADO · concluído em 05/10/2026 · QR do livro ES atualizados</t>
         </is>
       </c>
     </row>
@@ -943,10 +943,14 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>https://youtu.be/GSVU8n6kMvg</t>
+        </is>
+      </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>a subir</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -989,10 +993,14 @@
           <t>SIM (o original tem)</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>https://youtu.be/4GTcp9kH6jU</t>
+        </is>
+      </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>a subir</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1035,10 +1043,14 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>https://youtu.be/Tne_VzQ_WY4</t>
+        </is>
+      </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>a subir</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1081,10 +1093,14 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>https://youtu.be/iQxScbOixq4</t>
+        </is>
+      </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>a subir</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1127,10 +1143,14 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>https://youtu.be/sm7YdLUbpiM</t>
+        </is>
+      </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>a subir</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1173,10 +1193,14 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr"/>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>https://youtu.be/TI_NnU0IFrA</t>
+        </is>
+      </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>a subir</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1219,10 +1243,14 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>https://youtu.be/3VF4IdIZOPM</t>
+        </is>
+      </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>a subir</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1265,10 +1293,14 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="I18" s="6" t="inlineStr"/>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>https://youtu.be/xgXV0QI0FWY</t>
+        </is>
+      </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>a subir</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1311,10 +1343,14 @@
           <t>SIM (o original tem)</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr"/>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>https://youtu.be/kzvlkCbikmE</t>
+        </is>
+      </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>a subir</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1357,10 +1393,14 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr"/>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>https://youtu.be/0GK_Kpvh2JY</t>
+        </is>
+      </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>a subir</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1403,10 +1443,14 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="I21" s="6" t="inlineStr"/>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>https://youtu.be/acY8ePTK3fs</t>
+        </is>
+      </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>a subir</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1518,13 +1562,13 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>ver aba «Subir no YouTube»</t>
+          <t>https://youtu.be/GSVU8n6kMvg</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr"/>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>pronto</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1559,13 +1603,13 @@
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>ver aba «Subir no YouTube»</t>
+          <t>https://youtu.be/4GTcp9kH6jU</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr"/>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>pronto</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1600,13 +1644,13 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>ver aba «Subir no YouTube»</t>
+          <t>https://youtu.be/Tne_VzQ_WY4</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr"/>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>pronto</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1641,13 +1685,13 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>ver aba «Subir no YouTube»</t>
+          <t>https://youtu.be/iQxScbOixq4</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr"/>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>pronto</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1682,13 +1726,13 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>ver aba «Subir no YouTube»</t>
+          <t>https://youtu.be/sm7YdLUbpiM</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr"/>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>pronto</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1723,13 +1767,13 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>ver aba «Subir no YouTube»</t>
+          <t>https://youtu.be/TI_NnU0IFrA</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>pronto</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1764,13 +1808,13 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>ver aba «Subir no YouTube»</t>
+          <t>https://youtu.be/3VF4IdIZOPM</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr"/>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>pronto</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1805,13 +1849,13 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>ver aba «Subir no YouTube»</t>
+          <t>https://youtu.be/xgXV0QI0FWY</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>pronto</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1846,13 +1890,13 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>ver aba «Subir no YouTube»</t>
+          <t>https://youtu.be/kzvlkCbikmE</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr"/>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>pronto</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1887,13 +1931,13 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>ver aba «Subir no YouTube»</t>
+          <t>https://youtu.be/0GK_Kpvh2JY</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr"/>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>pronto</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -1928,13 +1972,13 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>ver aba «Subir no YouTube»</t>
+          <t>https://youtu.be/acY8ePTK3fs</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr"/>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>pronto</t>
+          <t>QR atualizado</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2152,7 @@
       <c r="H3" s="3" t="inlineStr"/>
       <c r="I3" s="8" t="inlineStr">
         <is>
-          <t>Regerar QR para a aula dublada quando o link ES existir</t>
+          <t>FEITO: QR regerado para a aula dublada no YouTube (não listada), conferido por escaneamento</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
@@ -2360,7 +2404,7 @@
       <c r="H8" s="3" t="inlineStr"/>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>Regerar QR para a aula dublada quando o link ES existir</t>
+          <t>FEITO: QR regerado para a aula dublada no YouTube (não listada), conferido por escaneamento</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
@@ -2456,7 +2500,7 @@
       <c r="H10" s="3" t="inlineStr"/>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>Regerar QR para a aula dublada quando o link ES existir</t>
+          <t>FEITO: QR regerado para a aula dublada no YouTube (não listada), conferido por escaneamento</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
@@ -2552,7 +2596,7 @@
       <c r="H12" s="3" t="inlineStr"/>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>Regerar QR para a aula dublada quando o link ES existir</t>
+          <t>FEITO: QR regerado para a aula dublada no YouTube (não listada), conferido por escaneamento</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
@@ -2648,7 +2692,7 @@
       <c r="H14" s="3" t="inlineStr"/>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>Regerar QR para a aula dublada quando o link ES existir</t>
+          <t>FEITO: QR regerado para a aula dublada no YouTube (não listada), conferido por escaneamento</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
@@ -2744,7 +2788,7 @@
       <c r="H16" s="3" t="inlineStr"/>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>Regerar QR para a aula dublada quando o link ES existir</t>
+          <t>FEITO: QR regerado para a aula dublada no YouTube (não listada), conferido por escaneamento</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
@@ -2788,7 +2832,7 @@
       <c r="H17" s="3" t="inlineStr"/>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>Regerar QR para a aula dublada quando o link ES existir</t>
+          <t>FEITO: QR regerado para a aula dublada no YouTube (não listada), conferido por escaneamento</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
@@ -2884,7 +2928,7 @@
       <c r="H19" s="3" t="inlineStr"/>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>Regerar QR para a aula dublada quando o link ES existir</t>
+          <t>FEITO: QR regerado para a aula dublada no YouTube (não listada), conferido por escaneamento</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
@@ -3032,7 +3076,7 @@
       <c r="H22" s="3" t="inlineStr"/>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>Regerar QR para a aula dublada quando o link ES existir</t>
+          <t>FEITO: QR regerado para a aula dublada no YouTube (não listada), conferido por escaneamento</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
@@ -3076,7 +3120,7 @@
       <c r="H23" s="3" t="inlineStr"/>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>Regerar QR para a aula dublada quando o link ES existir</t>
+          <t>FEITO: QR regerado para a aula dublada no YouTube (não listada), conferido por escaneamento</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
@@ -3120,7 +3164,7 @@
       <c r="H24" s="3" t="inlineStr"/>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>Regerar QR para a aula dublada quando o link ES existir</t>
+          <t>FEITO: QR regerado para a aula dublada no YouTube (não listada), conferido por escaneamento</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
@@ -3185,17 +3229,17 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Aulas dubladas</t>
+          <t>Corrigir os 6 QR com ERRO no PT</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Confirmar se as 11 aulas serão dubladas e publicadas no YouTube como não listadas, como no ebook de olheiras (18 aulas). A produção das aulas é da FEA, fora do escopo da skill.</t>
+          <t>Recomendação: corrigir o original PT (André) e eu aplico os mesmos destinos na versão ES. Os links propostos estão na aba «QR para ajustar».</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Keila</t>
+          <t>Keila + equipe médica</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -3208,17 +3252,17 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Corrigir os 6 QR com ERRO no PT</t>
+          <t>Numeração dos vídeos</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Recomendação: corrigir o original PT (André) e eu aplico os mesmos destinos na versão ES. Os links propostos estão na aba «QR para ajustar».</t>
+          <t>Só os 3 últimos boxes têm número (Vídeo 9, 10 e 11). Padronizar no ES: todos numerados ou nenhum. Recomendação: numerar todos de 1 a 11.</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Keila + equipe médica</t>
+          <t>Keila</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -3231,22 +3275,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Artigo da pág. 36</t>
+          <t>Título do livro em espanhol</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Subir o PDF do «Consensus Guidelines for the Management of Hyaluronic Acid Filler-Induced Vascular Occlusion» citado no box. Não existe no Drive.</t>
+          <t>Proposta: «Intercurrencias en el relleno con ácido hialurónico: diagnóstico y conductas clínicas ante complicaciones estéticas» (mantém «Intercurrencias», como na sigla ARTI do ebook de olheiras).</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Keila / equipe médica</t>
+          <t>Keila</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Só o QR da pág. 36</t>
+          <t>Não trava o PDF</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr"/>
@@ -3254,12 +3298,12 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Numeração dos vídeos</t>
+          <t>Compartilhamento dos artigos (conferido em 05/10)</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Só os 3 últimos boxes têm número (Vídeo 9, 10 e 11). Padronizar no ES: todos numerados ou nenhum. Recomendação: numerar todos de 1 a 11.</t>
+          <t>Só o artigo das págs. 23 e 61 abre para qualquer pessoa. Precisam de «Qualquer pessoa com o link: leitor» (Drive &gt; Compartilhar &gt; Acesso geral): Soares/Molecules (págs. 13, 30, 40) 1tHj3C58l9NhqokvQBIisp-RO25MrDGfp · HDPH DeLorenzi (pág. 18) 13rcR4MVX0frvJp3wgtFD1ko9IWQFiyco · Patterns (págs. 21, 26) 1F8aLFw8VV62JQngjfkHLNpHn2lr8jmjj · Hialuronidase (pág. 33) 19A8eYYAofI8Eiq4fIyk0kv-kJZf8aAvM · Kim JKMS (págs. 64, 68) 1DLM3QIm8ui-37tXlv33AazCSiK57hIgP.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -3269,7 +3313,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Não trava o PDF</t>
+          <t>Trava os QR de artigo (PT e ES)</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr"/>
@@ -3277,22 +3321,22 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Título do livro em espanhol</t>
+          <t>Artigo da pág. 36</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Proposta: «Intercurrencias en el relleno con ácido hialurónico: diagnóstico y conductas clínicas ante complicaciones estéticas» (mantém «Intercurrencias», como na sigla ARTI do ebook de olheiras).</t>
+          <t>O QR aponta para um arquivo que não existe mais. O box descreve o «Consensus Guidelines for the Management of HA Filler-Induced Vascular Occlusion»; o arquivo «2. ARTIGO delorenzi2014.pdf» do Drive é outro artigo (DeLorenzi, «Complications of Injectable Fillers, Part 2: Vascular Complications»). Ou sobe o Consensus, ou a equipe médica reescreve o box para o DeLorenzi 2014.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Keila</t>
+          <t>Equipe médica (Francine)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Não trava o PDF</t>
+          <t>Trava o QR da pág. 36</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr"/>

</xml_diff>